<commit_message>
Finalize dashboard pricing logic and configuration
</commit_message>
<xml_diff>
--- a/data/processed/apartment_base_prices.xlsx
+++ b/data/processed/apartment_base_prices.xlsx
@@ -511,10 +511,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>3487207.670698496</v>
+        <v>4283519.560704757</v>
       </c>
       <c r="K2" t="n">
-        <v>49254.34563133469</v>
+        <v>60501.68871051916</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>3307049.333733289</v>
+        <v>3957301.615367981</v>
       </c>
       <c r="K3" t="n">
-        <v>50412.33740447087</v>
+        <v>60324.71974646312</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -599,10 +599,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2839304.831580538</v>
+        <v>3395552.47607435</v>
       </c>
       <c r="K4" t="n">
-        <v>49812.36546632523</v>
+        <v>59571.09607147983</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>3702129.965534934</v>
+        <v>4337592.434186731</v>
       </c>
       <c r="K5" t="n">
-        <v>53654.05747152078</v>
+        <v>62863.65846647437</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -683,10 +683,10 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3702129.965534934</v>
+        <v>4337592.434186731</v>
       </c>
       <c r="K6" t="n">
-        <v>53654.05747152078</v>
+        <v>62863.65846647437</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>3702129.965534934</v>
+        <v>4337592.434186731</v>
       </c>
       <c r="K7" t="n">
-        <v>53654.05747152078</v>
+        <v>62863.65846647437</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -771,10 +771,10 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>5500300.237231525</v>
+        <v>7023172.797175091</v>
       </c>
       <c r="K8" t="n">
-        <v>49507.65290037376</v>
+        <v>63214.87666224204</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>3979414.761628558</v>
+        <v>4504586.904131437</v>
       </c>
       <c r="K9" t="n">
-        <v>57672.67770476171</v>
+        <v>65283.86817581792</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -855,10 +855,10 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3979414.761628558</v>
+        <v>4504586.904131437</v>
       </c>
       <c r="K10" t="n">
-        <v>57672.67770476171</v>
+        <v>65283.86817581792</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3979414.761628558</v>
+        <v>4504586.904131437</v>
       </c>
       <c r="K11" t="n">
-        <v>57672.67770476171</v>
+        <v>65283.86817581792</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -943,10 +943,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>5777585.03332515</v>
+        <v>7190167.267119796</v>
       </c>
       <c r="K12" t="n">
-        <v>52003.465646491</v>
+        <v>64717.97720179835</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -983,10 +983,10 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>4256699.557722183</v>
+        <v>4671581.374076141</v>
       </c>
       <c r="K13" t="n">
-        <v>61691.29793800265</v>
+        <v>67704.07788516146</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1023,10 +1023,10 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>4256699.557722183</v>
+        <v>4671581.374076141</v>
       </c>
       <c r="K14" t="n">
-        <v>61691.29793800265</v>
+        <v>67704.07788516146</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1063,10 +1063,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>4256699.557722183</v>
+        <v>4671581.374076141</v>
       </c>
       <c r="K15" t="n">
-        <v>61691.29793800265</v>
+        <v>67704.07788516146</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1107,10 +1107,10 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>6054869.829418774</v>
+        <v>7357161.7370645</v>
       </c>
       <c r="K16" t="n">
-        <v>54499.27839260823</v>
+        <v>66221.07774135465</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1147,10 +1147,10 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>4533984.353815807</v>
+        <v>4838575.844020846</v>
       </c>
       <c r="K17" t="n">
-        <v>65709.91817124358</v>
+        <v>70124.28759450502</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>4533984.353815807</v>
+        <v>4838575.844020846</v>
       </c>
       <c r="K18" t="n">
-        <v>65709.91817124358</v>
+        <v>70124.28759450502</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1235,10 +1235,10 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>4533984.353815807</v>
+        <v>4838575.844020846</v>
       </c>
       <c r="K19" t="n">
-        <v>65709.91817124358</v>
+        <v>70124.28759450502</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1279,10 +1279,10 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>6332154.625512399</v>
+        <v>7524156.207009205</v>
       </c>
       <c r="K20" t="n">
-        <v>56995.09113872547</v>
+        <v>67724.17828091094</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1323,10 +1323,10 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>4811269.149909432</v>
+        <v>5005570.313965551</v>
       </c>
       <c r="K21" t="n">
-        <v>69728.53840448453</v>
+        <v>72544.49730384856</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1363,10 +1363,10 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>4811269.149909432</v>
+        <v>5005570.313965551</v>
       </c>
       <c r="K22" t="n">
-        <v>69728.53840448453</v>
+        <v>72544.49730384856</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1407,10 +1407,10 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>4811269.149909432</v>
+        <v>5005570.313965551</v>
       </c>
       <c r="K23" t="n">
-        <v>69728.53840448453</v>
+        <v>72544.49730384856</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1451,10 +1451,10 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>6609439.421606023</v>
+        <v>7691150.67695391</v>
       </c>
       <c r="K24" t="n">
-        <v>59490.90388484269</v>
+        <v>69227.27882046724</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>5088553.946003056</v>
+        <v>5172564.783910255</v>
       </c>
       <c r="K25" t="n">
-        <v>73747.15863772546</v>
+        <v>74964.70701319211</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1535,10 +1535,10 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>5088553.946003056</v>
+        <v>5172564.783910255</v>
       </c>
       <c r="K26" t="n">
-        <v>73747.15863772546</v>
+        <v>74964.70701319211</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1579,10 +1579,10 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>5088553.946003056</v>
+        <v>5172564.783910255</v>
       </c>
       <c r="K27" t="n">
-        <v>73747.15863772546</v>
+        <v>74964.70701319211</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1623,10 +1623,10 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>6886724.217699647</v>
+        <v>7858145.146898614</v>
       </c>
       <c r="K28" t="n">
-        <v>61986.71663095992</v>
+        <v>70730.37936002354</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1663,10 +1663,10 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>5365838.742096681</v>
+        <v>5339559.253854959</v>
       </c>
       <c r="K29" t="n">
-        <v>77765.77887096639</v>
+        <v>77384.91672253564</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>5365838.742096681</v>
+        <v>5339559.253854959</v>
       </c>
       <c r="K30" t="n">
-        <v>77765.77887096639</v>
+        <v>77384.91672253564</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -1747,10 +1747,10 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>5365838.742096681</v>
+        <v>5339559.253854959</v>
       </c>
       <c r="K31" t="n">
-        <v>77765.77887096639</v>
+        <v>77384.91672253564</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -1791,10 +1791,10 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>7164009.013793272</v>
+        <v>8025139.616843319</v>
       </c>
       <c r="K32" t="n">
-        <v>64482.52937707716</v>
+        <v>72233.47989957983</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -1831,10 +1831,10 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>5643123.538190305</v>
+        <v>5506553.723799665</v>
       </c>
       <c r="K33" t="n">
-        <v>81784.39910420732</v>
+        <v>79805.12643187919</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -1871,10 +1871,10 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>5643123.538190305</v>
+        <v>5506553.723799665</v>
       </c>
       <c r="K34" t="n">
-        <v>81784.39910420732</v>
+        <v>79805.12643187919</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -1911,10 +1911,10 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>5643123.538190305</v>
+        <v>5506553.723799665</v>
       </c>
       <c r="K35" t="n">
-        <v>81784.39910420732</v>
+        <v>79805.12643187919</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -1955,10 +1955,10 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>7441293.809886897</v>
+        <v>8192134.086788024</v>
       </c>
       <c r="K36" t="n">
-        <v>66978.34212319439</v>
+        <v>73736.58043913613</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -1999,10 +1999,10 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>12880833.6194382</v>
+        <v>17421364.54085964</v>
       </c>
       <c r="K37" t="n">
-        <v>50473.48596958544</v>
+        <v>68265.53503471646</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2043,10 +2043,10 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>13050598.20619388</v>
+        <v>17728762.2201193</v>
       </c>
       <c r="K38" t="n">
-        <v>50175.31028909604</v>
+        <v>68161.33110388041</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2087,10 +2087,10 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>10102263.47281404</v>
+        <v>12104917.24206561</v>
       </c>
       <c r="K39" t="n">
-        <v>59390.14387309841</v>
+        <v>71163.53463883368</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2127,10 +2127,10 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>9364255.722489629</v>
+        <v>11339004.01894366</v>
       </c>
       <c r="K40" t="n">
-        <v>59043.22649741254</v>
+        <v>71494.35068690831</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>

</xml_diff>